<commit_message>
Ajuste: removendo temp_inputs e correção do app
</commit_message>
<xml_diff>
--- a/exit/Meta49_preenchido.xlsx
+++ b/exit/Meta49_preenchido.xlsx
@@ -464,7 +464,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -774,10 +774,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="21" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="21" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="22" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="23" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12899,7 +12895,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D4" s="145" t="n">
+      <c r="D4" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="116" t="n"/>
@@ -12913,7 +12909,7 @@
       <c r="M4" s="116" t="n"/>
       <c r="N4" s="116" t="n"/>
       <c r="O4" s="116" t="n"/>
-      <c r="P4" s="145" t="n">
+      <c r="P4" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12933,7 +12929,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D5" s="146" t="n">
+      <c r="D5" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="119" t="n"/>
@@ -12947,7 +12943,7 @@
       <c r="M5" s="119" t="n"/>
       <c r="N5" s="119" t="n"/>
       <c r="O5" s="119" t="n"/>
-      <c r="P5" s="147" t="n">
+      <c r="P5" s="120" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12967,7 +12963,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D6" s="146" t="n">
+      <c r="D6" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="119" t="n"/>
@@ -12981,7 +12977,7 @@
       <c r="M6" s="119" t="n"/>
       <c r="N6" s="119" t="n"/>
       <c r="O6" s="119" t="n"/>
-      <c r="P6" s="146" t="n">
+      <c r="P6" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13001,7 +12997,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D7" s="145" t="n">
+      <c r="D7" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="116" t="n"/>
@@ -13015,7 +13011,7 @@
       <c r="M7" s="116" t="n"/>
       <c r="N7" s="116" t="n"/>
       <c r="O7" s="116" t="n"/>
-      <c r="P7" s="145" t="n">
+      <c r="P7" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13035,7 +13031,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D8" s="146" t="n">
+      <c r="D8" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="119" t="n"/>
@@ -13049,7 +13045,7 @@
       <c r="M8" s="119" t="n"/>
       <c r="N8" s="119" t="n"/>
       <c r="O8" s="119" t="n"/>
-      <c r="P8" s="146" t="n">
+      <c r="P8" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13069,7 +13065,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D9" s="146" t="n">
+      <c r="D9" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="119" t="n"/>
@@ -13083,7 +13079,7 @@
       <c r="M9" s="119" t="n"/>
       <c r="N9" s="119" t="n"/>
       <c r="O9" s="119" t="n"/>
-      <c r="P9" s="146" t="n">
+      <c r="P9" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13103,7 +13099,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D10" s="145" t="n">
+      <c r="D10" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="116" t="n"/>
@@ -13117,7 +13113,7 @@
       <c r="M10" s="116" t="n"/>
       <c r="N10" s="116" t="n"/>
       <c r="O10" s="116" t="n"/>
-      <c r="P10" s="145" t="n">
+      <c r="P10" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13137,7 +13133,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D11" s="146" t="n">
+      <c r="D11" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="119" t="n"/>
@@ -13151,7 +13147,7 @@
       <c r="M11" s="119" t="n"/>
       <c r="N11" s="119" t="n"/>
       <c r="O11" s="119" t="n"/>
-      <c r="P11" s="146" t="n">
+      <c r="P11" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13171,7 +13167,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D12" s="146" t="n">
+      <c r="D12" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="119" t="n"/>
@@ -13185,7 +13181,7 @@
       <c r="M12" s="119" t="n"/>
       <c r="N12" s="119" t="n"/>
       <c r="O12" s="119" t="n"/>
-      <c r="P12" s="146" t="n">
+      <c r="P12" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13205,7 +13201,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D13" s="145" t="n">
+      <c r="D13" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="116" t="n"/>
@@ -13219,7 +13215,7 @@
       <c r="M13" s="116" t="n"/>
       <c r="N13" s="116" t="n"/>
       <c r="O13" s="116" t="n"/>
-      <c r="P13" s="145" t="n">
+      <c r="P13" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13239,7 +13235,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D14" s="146" t="n">
+      <c r="D14" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="119" t="n"/>
@@ -13253,7 +13249,7 @@
       <c r="M14" s="119" t="n"/>
       <c r="N14" s="119" t="n"/>
       <c r="O14" s="119" t="n"/>
-      <c r="P14" s="146" t="n">
+      <c r="P14" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13273,7 +13269,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D15" s="146" t="n">
+      <c r="D15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="119" t="n"/>
@@ -13287,7 +13283,7 @@
       <c r="M15" s="119" t="n"/>
       <c r="N15" s="119" t="n"/>
       <c r="O15" s="119" t="n"/>
-      <c r="P15" s="146" t="n">
+      <c r="P15" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13307,7 +13303,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D16" s="145" t="n">
+      <c r="D16" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="116" t="n"/>
@@ -13321,7 +13317,7 @@
       <c r="M16" s="116" t="n"/>
       <c r="N16" s="116" t="n"/>
       <c r="O16" s="116" t="n"/>
-      <c r="P16" s="145" t="n">
+      <c r="P16" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13341,7 +13337,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D17" s="146" t="n">
+      <c r="D17" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="119" t="n"/>
@@ -13355,7 +13351,7 @@
       <c r="M17" s="119" t="n"/>
       <c r="N17" s="119" t="n"/>
       <c r="O17" s="119" t="n"/>
-      <c r="P17" s="146" t="n">
+      <c r="P17" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13375,7 +13371,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D18" s="146" t="n">
+      <c r="D18" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="119" t="n"/>
@@ -13389,7 +13385,7 @@
       <c r="M18" s="119" t="n"/>
       <c r="N18" s="119" t="n"/>
       <c r="O18" s="119" t="n"/>
-      <c r="P18" s="146" t="n">
+      <c r="P18" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13409,7 +13405,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D19" s="145" t="n">
+      <c r="D19" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="116" t="n"/>
@@ -13423,7 +13419,7 @@
       <c r="M19" s="116" t="n"/>
       <c r="N19" s="116" t="n"/>
       <c r="O19" s="116" t="n"/>
-      <c r="P19" s="145" t="n">
+      <c r="P19" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13443,7 +13439,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D20" s="146" t="n">
+      <c r="D20" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="119" t="n"/>
@@ -13457,7 +13453,7 @@
       <c r="M20" s="119" t="n"/>
       <c r="N20" s="119" t="n"/>
       <c r="O20" s="119" t="n"/>
-      <c r="P20" s="146" t="n">
+      <c r="P20" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13477,7 +13473,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D21" s="146" t="n">
+      <c r="D21" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="119" t="n"/>
@@ -13491,7 +13487,7 @@
       <c r="M21" s="119" t="n"/>
       <c r="N21" s="119" t="n"/>
       <c r="O21" s="119" t="n"/>
-      <c r="P21" s="146" t="n">
+      <c r="P21" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13511,7 +13507,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D22" s="145" t="n">
+      <c r="D22" s="116" t="n">
         <v>17631</v>
       </c>
       <c r="E22" s="116" t="n"/>
@@ -13525,7 +13521,7 @@
       <c r="M22" s="116" t="n"/>
       <c r="N22" s="116" t="n"/>
       <c r="O22" s="116" t="n"/>
-      <c r="P22" s="145" t="n">
+      <c r="P22" s="116" t="n">
         <v>17631</v>
       </c>
     </row>
@@ -13545,7 +13541,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D23" s="146" t="n">
+      <c r="D23" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="119" t="n"/>
@@ -13559,7 +13555,7 @@
       <c r="M23" s="119" t="n"/>
       <c r="N23" s="119" t="n"/>
       <c r="O23" s="119" t="n"/>
-      <c r="P23" s="146" t="n">
+      <c r="P23" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13579,7 +13575,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D24" s="146" t="n">
+      <c r="D24" s="119" t="n">
         <v>17631</v>
       </c>
       <c r="E24" s="119" t="n"/>
@@ -13593,7 +13589,7 @@
       <c r="M24" s="119" t="n"/>
       <c r="N24" s="119" t="n"/>
       <c r="O24" s="119" t="n"/>
-      <c r="P24" s="146" t="n">
+      <c r="P24" s="119" t="n">
         <v>17631</v>
       </c>
     </row>
@@ -13613,7 +13609,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D25" s="145" t="n">
+      <c r="D25" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="116" t="n"/>
@@ -13627,7 +13623,7 @@
       <c r="M25" s="116" t="n"/>
       <c r="N25" s="116" t="n"/>
       <c r="O25" s="116" t="n"/>
-      <c r="P25" s="145" t="n">
+      <c r="P25" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13647,7 +13643,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D26" s="146" t="n">
+      <c r="D26" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="119" t="n"/>
@@ -13661,7 +13657,7 @@
       <c r="M26" s="119" t="n"/>
       <c r="N26" s="119" t="n"/>
       <c r="O26" s="119" t="n"/>
-      <c r="P26" s="146" t="n">
+      <c r="P26" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13681,7 +13677,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D27" s="146" t="n">
+      <c r="D27" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="119" t="n"/>
@@ -13695,7 +13691,7 @@
       <c r="M27" s="119" t="n"/>
       <c r="N27" s="119" t="n"/>
       <c r="O27" s="119" t="n"/>
-      <c r="P27" s="146" t="n">
+      <c r="P27" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13715,7 +13711,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D28" s="145" t="n">
+      <c r="D28" s="116" t="n">
         <v>2840.1</v>
       </c>
       <c r="E28" s="116" t="n"/>
@@ -13729,7 +13725,7 @@
       <c r="M28" s="116" t="n"/>
       <c r="N28" s="116" t="n"/>
       <c r="O28" s="116" t="n"/>
-      <c r="P28" s="145" t="n">
+      <c r="P28" s="116" t="n">
         <v>2840.1</v>
       </c>
     </row>
@@ -13749,7 +13745,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D29" s="146" t="n">
+      <c r="D29" s="119" t="n">
         <v>2840.1</v>
       </c>
       <c r="E29" s="119" t="n"/>
@@ -13763,7 +13759,7 @@
       <c r="M29" s="119" t="n"/>
       <c r="N29" s="119" t="n"/>
       <c r="O29" s="119" t="n"/>
-      <c r="P29" s="146" t="n">
+      <c r="P29" s="119" t="n">
         <v>2840.1</v>
       </c>
     </row>
@@ -13783,7 +13779,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D30" s="146" t="n">
+      <c r="D30" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="119" t="n"/>
@@ -13797,7 +13793,7 @@
       <c r="M30" s="119" t="n"/>
       <c r="N30" s="119" t="n"/>
       <c r="O30" s="119" t="n"/>
-      <c r="P30" s="146" t="n">
+      <c r="P30" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13817,7 +13813,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D31" s="145" t="n">
+      <c r="D31" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="116" t="n"/>
@@ -13831,7 +13827,7 @@
       <c r="M31" s="116" t="n"/>
       <c r="N31" s="116" t="n"/>
       <c r="O31" s="116" t="n"/>
-      <c r="P31" s="145" t="n">
+      <c r="P31" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13851,7 +13847,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D32" s="146" t="n">
+      <c r="D32" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="119" t="n"/>
@@ -13865,7 +13861,7 @@
       <c r="M32" s="119" t="n"/>
       <c r="N32" s="119" t="n"/>
       <c r="O32" s="119" t="n"/>
-      <c r="P32" s="146" t="n">
+      <c r="P32" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13885,7 +13881,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D33" s="146" t="n">
+      <c r="D33" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="119" t="n"/>
@@ -13899,7 +13895,7 @@
       <c r="M33" s="119" t="n"/>
       <c r="N33" s="119" t="n"/>
       <c r="O33" s="119" t="n"/>
-      <c r="P33" s="146" t="n">
+      <c r="P33" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13919,7 +13915,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D34" s="145" t="n">
+      <c r="D34" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="116" t="n"/>
@@ -13933,7 +13929,7 @@
       <c r="M34" s="116" t="n"/>
       <c r="N34" s="116" t="n"/>
       <c r="O34" s="116" t="n"/>
-      <c r="P34" s="145" t="n">
+      <c r="P34" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13953,7 +13949,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D35" s="146" t="n">
+      <c r="D35" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="119" t="n"/>
@@ -13967,7 +13963,7 @@
       <c r="M35" s="119" t="n"/>
       <c r="N35" s="119" t="n"/>
       <c r="O35" s="119" t="n"/>
-      <c r="P35" s="146" t="n">
+      <c r="P35" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13987,7 +13983,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D36" s="146" t="n">
+      <c r="D36" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="119" t="n"/>
@@ -14001,7 +13997,7 @@
       <c r="M36" s="119" t="n"/>
       <c r="N36" s="119" t="n"/>
       <c r="O36" s="119" t="n"/>
-      <c r="P36" s="146" t="n">
+      <c r="P36" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14021,7 +14017,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D37" s="145" t="n">
+      <c r="D37" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="116" t="n"/>
@@ -14035,7 +14031,7 @@
       <c r="M37" s="116" t="n"/>
       <c r="N37" s="116" t="n"/>
       <c r="O37" s="116" t="n"/>
-      <c r="P37" s="145" t="n">
+      <c r="P37" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14055,7 +14051,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D38" s="146" t="n">
+      <c r="D38" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E38" s="119" t="n"/>
@@ -14069,7 +14065,7 @@
       <c r="M38" s="119" t="n"/>
       <c r="N38" s="119" t="n"/>
       <c r="O38" s="119" t="n"/>
-      <c r="P38" s="146" t="n">
+      <c r="P38" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14089,7 +14085,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D39" s="146" t="n">
+      <c r="D39" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E39" s="119" t="n"/>
@@ -14103,7 +14099,7 @@
       <c r="M39" s="119" t="n"/>
       <c r="N39" s="119" t="n"/>
       <c r="O39" s="119" t="n"/>
-      <c r="P39" s="146" t="n">
+      <c r="P39" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14123,7 +14119,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D40" s="145" t="n">
+      <c r="D40" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E40" s="116" t="n"/>
@@ -14137,7 +14133,7 @@
       <c r="M40" s="116" t="n"/>
       <c r="N40" s="116" t="n"/>
       <c r="O40" s="116" t="n"/>
-      <c r="P40" s="145" t="n">
+      <c r="P40" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14157,7 +14153,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D41" s="146" t="n">
+      <c r="D41" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E41" s="119" t="n"/>
@@ -14171,7 +14167,7 @@
       <c r="M41" s="119" t="n"/>
       <c r="N41" s="119" t="n"/>
       <c r="O41" s="119" t="n"/>
-      <c r="P41" s="146" t="n">
+      <c r="P41" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14191,7 +14187,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D42" s="146" t="n">
+      <c r="D42" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="119" t="n"/>
@@ -14205,7 +14201,7 @@
       <c r="M42" s="119" t="n"/>
       <c r="N42" s="119" t="n"/>
       <c r="O42" s="119" t="n"/>
-      <c r="P42" s="146" t="n">
+      <c r="P42" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14225,7 +14221,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D43" s="145" t="n">
+      <c r="D43" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="116" t="n"/>
@@ -14239,7 +14235,7 @@
       <c r="M43" s="116" t="n"/>
       <c r="N43" s="116" t="n"/>
       <c r="O43" s="116" t="n"/>
-      <c r="P43" s="145" t="n">
+      <c r="P43" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14259,7 +14255,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D44" s="146" t="n">
+      <c r="D44" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="119" t="n"/>
@@ -14273,7 +14269,7 @@
       <c r="M44" s="119" t="n"/>
       <c r="N44" s="119" t="n"/>
       <c r="O44" s="119" t="n"/>
-      <c r="P44" s="146" t="n">
+      <c r="P44" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14293,7 +14289,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D45" s="146" t="n">
+      <c r="D45" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="119" t="n"/>
@@ -14307,7 +14303,7 @@
       <c r="M45" s="119" t="n"/>
       <c r="N45" s="119" t="n"/>
       <c r="O45" s="119" t="n"/>
-      <c r="P45" s="146" t="n">
+      <c r="P45" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14327,7 +14323,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D46" s="145" t="n">
+      <c r="D46" s="116" t="n">
         <v>16322.7</v>
       </c>
       <c r="E46" s="116" t="n"/>
@@ -14341,7 +14337,7 @@
       <c r="M46" s="116" t="n"/>
       <c r="N46" s="116" t="n"/>
       <c r="O46" s="116" t="n"/>
-      <c r="P46" s="145" t="n">
+      <c r="P46" s="116" t="n">
         <v>16322.7</v>
       </c>
     </row>
@@ -14361,7 +14357,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D47" s="146" t="n">
+      <c r="D47" s="119" t="n">
         <v>2897.7</v>
       </c>
       <c r="E47" s="119" t="n"/>
@@ -14375,7 +14371,7 @@
       <c r="M47" s="119" t="n"/>
       <c r="N47" s="119" t="n"/>
       <c r="O47" s="119" t="n"/>
-      <c r="P47" s="146" t="n">
+      <c r="P47" s="119" t="n">
         <v>2897.7</v>
       </c>
     </row>
@@ -14395,7 +14391,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D48" s="146" t="n">
+      <c r="D48" s="119" t="n">
         <v>13425</v>
       </c>
       <c r="E48" s="119" t="n"/>
@@ -14409,7 +14405,7 @@
       <c r="M48" s="119" t="n"/>
       <c r="N48" s="119" t="n"/>
       <c r="O48" s="119" t="n"/>
-      <c r="P48" s="146" t="n">
+      <c r="P48" s="119" t="n">
         <v>13425</v>
       </c>
     </row>
@@ -14429,7 +14425,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D49" s="145" t="n">
+      <c r="D49" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="116" t="n"/>
@@ -14443,7 +14439,7 @@
       <c r="M49" s="116" t="n"/>
       <c r="N49" s="116" t="n"/>
       <c r="O49" s="116" t="n"/>
-      <c r="P49" s="145" t="n">
+      <c r="P49" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14463,7 +14459,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D50" s="146" t="n">
+      <c r="D50" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E50" s="119" t="n"/>
@@ -14477,7 +14473,7 @@
       <c r="M50" s="119" t="n"/>
       <c r="N50" s="119" t="n"/>
       <c r="O50" s="119" t="n"/>
-      <c r="P50" s="146" t="n">
+      <c r="P50" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14497,7 +14493,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D51" s="146" t="n">
+      <c r="D51" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E51" s="119" t="n"/>
@@ -14511,7 +14507,7 @@
       <c r="M51" s="119" t="n"/>
       <c r="N51" s="119" t="n"/>
       <c r="O51" s="119" t="n"/>
-      <c r="P51" s="146" t="n">
+      <c r="P51" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14531,7 +14527,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D52" s="145" t="n">
+      <c r="D52" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E52" s="116" t="n"/>
@@ -14545,7 +14541,7 @@
       <c r="M52" s="116" t="n"/>
       <c r="N52" s="116" t="n"/>
       <c r="O52" s="116" t="n"/>
-      <c r="P52" s="145" t="n">
+      <c r="P52" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14565,7 +14561,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D53" s="146" t="n">
+      <c r="D53" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E53" s="119" t="n"/>
@@ -14579,7 +14575,7 @@
       <c r="M53" s="119" t="n"/>
       <c r="N53" s="119" t="n"/>
       <c r="O53" s="119" t="n"/>
-      <c r="P53" s="146" t="n">
+      <c r="P53" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14599,7 +14595,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D54" s="146" t="n">
+      <c r="D54" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="119" t="n"/>
@@ -14613,7 +14609,7 @@
       <c r="M54" s="119" t="n"/>
       <c r="N54" s="119" t="n"/>
       <c r="O54" s="119" t="n"/>
-      <c r="P54" s="146" t="n">
+      <c r="P54" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14633,7 +14629,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D55" s="145" t="n">
+      <c r="D55" s="116" t="n">
         <v>1066</v>
       </c>
       <c r="E55" s="116" t="n"/>
@@ -14647,7 +14643,7 @@
       <c r="M55" s="116" t="n"/>
       <c r="N55" s="116" t="n"/>
       <c r="O55" s="116" t="n"/>
-      <c r="P55" s="145" t="n">
+      <c r="P55" s="116" t="n">
         <v>1066</v>
       </c>
     </row>
@@ -14667,7 +14663,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D56" s="146" t="n">
+      <c r="D56" s="119" t="n">
         <v>1066</v>
       </c>
       <c r="E56" s="119" t="n"/>
@@ -14681,7 +14677,7 @@
       <c r="M56" s="119" t="n"/>
       <c r="N56" s="119" t="n"/>
       <c r="O56" s="119" t="n"/>
-      <c r="P56" s="146" t="n">
+      <c r="P56" s="119" t="n">
         <v>1066</v>
       </c>
     </row>
@@ -14701,7 +14697,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D57" s="146" t="n">
+      <c r="D57" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="119" t="n"/>
@@ -14715,7 +14711,7 @@
       <c r="M57" s="119" t="n"/>
       <c r="N57" s="119" t="n"/>
       <c r="O57" s="119" t="n"/>
-      <c r="P57" s="146" t="n">
+      <c r="P57" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14735,7 +14731,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D58" s="145" t="n">
+      <c r="D58" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E58" s="116" t="n"/>
@@ -14749,7 +14745,7 @@
       <c r="M58" s="116" t="n"/>
       <c r="N58" s="116" t="n"/>
       <c r="O58" s="116" t="n"/>
-      <c r="P58" s="145" t="n">
+      <c r="P58" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14769,7 +14765,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D59" s="146" t="n">
+      <c r="D59" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E59" s="119" t="n"/>
@@ -14783,7 +14779,7 @@
       <c r="M59" s="119" t="n"/>
       <c r="N59" s="119" t="n"/>
       <c r="O59" s="119" t="n"/>
-      <c r="P59" s="146" t="n">
+      <c r="P59" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14803,7 +14799,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D60" s="146" t="n">
+      <c r="D60" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="119" t="n"/>
@@ -14817,7 +14813,7 @@
       <c r="M60" s="119" t="n"/>
       <c r="N60" s="119" t="n"/>
       <c r="O60" s="119" t="n"/>
-      <c r="P60" s="146" t="n">
+      <c r="P60" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14837,7 +14833,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D61" s="145" t="n">
+      <c r="D61" s="116" t="n">
         <v>7912.81</v>
       </c>
       <c r="E61" s="116" t="n"/>
@@ -14851,7 +14847,7 @@
       <c r="M61" s="116" t="n"/>
       <c r="N61" s="116" t="n"/>
       <c r="O61" s="116" t="n"/>
-      <c r="P61" s="145" t="n">
+      <c r="P61" s="116" t="n">
         <v>7912.81</v>
       </c>
     </row>
@@ -14871,7 +14867,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D62" s="146" t="n">
+      <c r="D62" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E62" s="119" t="n"/>
@@ -14885,7 +14881,7 @@
       <c r="M62" s="119" t="n"/>
       <c r="N62" s="119" t="n"/>
       <c r="O62" s="119" t="n"/>
-      <c r="P62" s="146" t="n">
+      <c r="P62" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14905,7 +14901,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D63" s="146" t="n">
+      <c r="D63" s="119" t="n">
         <v>7912.81</v>
       </c>
       <c r="E63" s="119" t="n"/>
@@ -14919,7 +14915,7 @@
       <c r="M63" s="119" t="n"/>
       <c r="N63" s="119" t="n"/>
       <c r="O63" s="119" t="n"/>
-      <c r="P63" s="146" t="n">
+      <c r="P63" s="119" t="n">
         <v>7912.81</v>
       </c>
     </row>
@@ -14939,7 +14935,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D64" s="145" t="n">
+      <c r="D64" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E64" s="116" t="n"/>
@@ -14953,7 +14949,7 @@
       <c r="M64" s="116" t="n"/>
       <c r="N64" s="116" t="n"/>
       <c r="O64" s="116" t="n"/>
-      <c r="P64" s="145" t="n">
+      <c r="P64" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14973,7 +14969,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D65" s="146" t="n">
+      <c r="D65" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E65" s="119" t="n"/>
@@ -14987,7 +14983,7 @@
       <c r="M65" s="119" t="n"/>
       <c r="N65" s="119" t="n"/>
       <c r="O65" s="119" t="n"/>
-      <c r="P65" s="146" t="n">
+      <c r="P65" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15007,7 +15003,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D66" s="146" t="n">
+      <c r="D66" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E66" s="119" t="n"/>
@@ -15021,7 +15017,7 @@
       <c r="M66" s="119" t="n"/>
       <c r="N66" s="119" t="n"/>
       <c r="O66" s="119" t="n"/>
-      <c r="P66" s="146" t="n">
+      <c r="P66" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15041,7 +15037,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D67" s="145" t="n">
+      <c r="D67" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E67" s="116" t="n"/>
@@ -15055,7 +15051,7 @@
       <c r="M67" s="116" t="n"/>
       <c r="N67" s="116" t="n"/>
       <c r="O67" s="116" t="n"/>
-      <c r="P67" s="145" t="n">
+      <c r="P67" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15075,7 +15071,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D68" s="146" t="n">
+      <c r="D68" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E68" s="119" t="n"/>
@@ -15089,7 +15085,7 @@
       <c r="M68" s="119" t="n"/>
       <c r="N68" s="119" t="n"/>
       <c r="O68" s="119" t="n"/>
-      <c r="P68" s="146" t="n">
+      <c r="P68" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15109,7 +15105,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D69" s="146" t="n">
+      <c r="D69" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E69" s="119" t="n"/>
@@ -15123,7 +15119,7 @@
       <c r="M69" s="119" t="n"/>
       <c r="N69" s="119" t="n"/>
       <c r="O69" s="119" t="n"/>
-      <c r="P69" s="146" t="n">
+      <c r="P69" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15143,7 +15139,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D70" s="145" t="n">
+      <c r="D70" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E70" s="116" t="n"/>
@@ -15157,7 +15153,7 @@
       <c r="M70" s="116" t="n"/>
       <c r="N70" s="116" t="n"/>
       <c r="O70" s="116" t="n"/>
-      <c r="P70" s="145" t="n">
+      <c r="P70" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15177,7 +15173,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D71" s="146" t="n">
+      <c r="D71" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E71" s="119" t="n"/>
@@ -15191,7 +15187,7 @@
       <c r="M71" s="119" t="n"/>
       <c r="N71" s="119" t="n"/>
       <c r="O71" s="119" t="n"/>
-      <c r="P71" s="146" t="n">
+      <c r="P71" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15211,7 +15207,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D72" s="146" t="n">
+      <c r="D72" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E72" s="119" t="n"/>
@@ -15225,7 +15221,7 @@
       <c r="M72" s="119" t="n"/>
       <c r="N72" s="119" t="n"/>
       <c r="O72" s="119" t="n"/>
-      <c r="P72" s="146" t="n">
+      <c r="P72" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15245,7 +15241,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D73" s="145" t="n">
+      <c r="D73" s="116" t="n">
         <v>3041.3</v>
       </c>
       <c r="E73" s="116" t="n"/>
@@ -15259,7 +15255,7 @@
       <c r="M73" s="116" t="n"/>
       <c r="N73" s="116" t="n"/>
       <c r="O73" s="116" t="n"/>
-      <c r="P73" s="145" t="n">
+      <c r="P73" s="116" t="n">
         <v>3041.3</v>
       </c>
     </row>
@@ -15279,7 +15275,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D74" s="146" t="n">
+      <c r="D74" s="119" t="n">
         <v>3041.3</v>
       </c>
       <c r="E74" s="119" t="n"/>
@@ -15293,7 +15289,7 @@
       <c r="M74" s="119" t="n"/>
       <c r="N74" s="119" t="n"/>
       <c r="O74" s="119" t="n"/>
-      <c r="P74" s="146" t="n">
+      <c r="P74" s="119" t="n">
         <v>3041.3</v>
       </c>
     </row>
@@ -15313,7 +15309,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D75" s="146" t="n">
+      <c r="D75" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E75" s="119" t="n"/>
@@ -15327,7 +15323,7 @@
       <c r="M75" s="119" t="n"/>
       <c r="N75" s="119" t="n"/>
       <c r="O75" s="119" t="n"/>
-      <c r="P75" s="146" t="n">
+      <c r="P75" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15347,7 +15343,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D76" s="145" t="n">
+      <c r="D76" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E76" s="116" t="n"/>
@@ -15361,7 +15357,7 @@
       <c r="M76" s="116" t="n"/>
       <c r="N76" s="116" t="n"/>
       <c r="O76" s="116" t="n"/>
-      <c r="P76" s="145" t="n">
+      <c r="P76" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15381,7 +15377,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D77" s="146" t="n">
+      <c r="D77" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E77" s="119" t="n"/>
@@ -15395,7 +15391,7 @@
       <c r="M77" s="119" t="n"/>
       <c r="N77" s="119" t="n"/>
       <c r="O77" s="119" t="n"/>
-      <c r="P77" s="146" t="n">
+      <c r="P77" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15415,7 +15411,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D78" s="146" t="n">
+      <c r="D78" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E78" s="119" t="n"/>
@@ -15429,7 +15425,7 @@
       <c r="M78" s="119" t="n"/>
       <c r="N78" s="119" t="n"/>
       <c r="O78" s="119" t="n"/>
-      <c r="P78" s="146" t="n">
+      <c r="P78" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15449,7 +15445,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D79" s="145" t="n">
+      <c r="D79" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E79" s="116" t="n"/>
@@ -15463,7 +15459,7 @@
       <c r="M79" s="116" t="n"/>
       <c r="N79" s="116" t="n"/>
       <c r="O79" s="116" t="n"/>
-      <c r="P79" s="145" t="n">
+      <c r="P79" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15483,7 +15479,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D80" s="146" t="n">
+      <c r="D80" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E80" s="119" t="n"/>
@@ -15497,7 +15493,7 @@
       <c r="M80" s="119" t="n"/>
       <c r="N80" s="119" t="n"/>
       <c r="O80" s="119" t="n"/>
-      <c r="P80" s="146" t="n">
+      <c r="P80" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15517,7 +15513,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D81" s="146" t="n">
+      <c r="D81" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E81" s="119" t="n"/>
@@ -15531,7 +15527,7 @@
       <c r="M81" s="119" t="n"/>
       <c r="N81" s="119" t="n"/>
       <c r="O81" s="119" t="n"/>
-      <c r="P81" s="146" t="n">
+      <c r="P81" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15551,7 +15547,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D82" s="145" t="n">
+      <c r="D82" s="116" t="n">
         <v>2546</v>
       </c>
       <c r="E82" s="116" t="n"/>
@@ -15565,7 +15561,7 @@
       <c r="M82" s="116" t="n"/>
       <c r="N82" s="116" t="n"/>
       <c r="O82" s="116" t="n"/>
-      <c r="P82" s="145" t="n">
+      <c r="P82" s="116" t="n">
         <v>2546</v>
       </c>
     </row>
@@ -15585,7 +15581,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D83" s="146" t="n">
+      <c r="D83" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E83" s="119" t="n"/>
@@ -15599,7 +15595,7 @@
       <c r="M83" s="119" t="n"/>
       <c r="N83" s="119" t="n"/>
       <c r="O83" s="119" t="n"/>
-      <c r="P83" s="146" t="n">
+      <c r="P83" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15619,7 +15615,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D84" s="146" t="n">
+      <c r="D84" s="119" t="n">
         <v>2546</v>
       </c>
       <c r="E84" s="119" t="n"/>
@@ -15633,7 +15629,7 @@
       <c r="M84" s="119" t="n"/>
       <c r="N84" s="119" t="n"/>
       <c r="O84" s="119" t="n"/>
-      <c r="P84" s="146" t="n">
+      <c r="P84" s="119" t="n">
         <v>2546</v>
       </c>
     </row>
@@ -15653,7 +15649,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D85" s="145" t="n">
+      <c r="D85" s="116" t="n">
         <v>6924</v>
       </c>
       <c r="E85" s="116" t="n"/>
@@ -15667,7 +15663,7 @@
       <c r="M85" s="116" t="n"/>
       <c r="N85" s="116" t="n"/>
       <c r="O85" s="116" t="n"/>
-      <c r="P85" s="145" t="n">
+      <c r="P85" s="116" t="n">
         <v>6924</v>
       </c>
     </row>
@@ -15687,7 +15683,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D86" s="146" t="n">
+      <c r="D86" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E86" s="119" t="n"/>
@@ -15701,7 +15697,7 @@
       <c r="M86" s="119" t="n"/>
       <c r="N86" s="119" t="n"/>
       <c r="O86" s="119" t="n"/>
-      <c r="P86" s="146" t="n">
+      <c r="P86" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15721,7 +15717,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D87" s="146" t="n">
+      <c r="D87" s="119" t="n">
         <v>6924</v>
       </c>
       <c r="E87" s="119" t="n"/>
@@ -15735,7 +15731,7 @@
       <c r="M87" s="119" t="n"/>
       <c r="N87" s="119" t="n"/>
       <c r="O87" s="119" t="n"/>
-      <c r="P87" s="146" t="n">
+      <c r="P87" s="119" t="n">
         <v>6924</v>
       </c>
     </row>
@@ -15755,7 +15751,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D88" s="145" t="n">
+      <c r="D88" s="116" t="n">
         <v>4269.55</v>
       </c>
       <c r="E88" s="116" t="n"/>
@@ -15769,7 +15765,7 @@
       <c r="M88" s="116" t="n"/>
       <c r="N88" s="116" t="n"/>
       <c r="O88" s="116" t="n"/>
-      <c r="P88" s="145" t="n">
+      <c r="P88" s="116" t="n">
         <v>4269.55</v>
       </c>
     </row>
@@ -15789,7 +15785,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D89" s="146" t="n">
+      <c r="D89" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E89" s="119" t="n"/>
@@ -15803,7 +15799,7 @@
       <c r="M89" s="119" t="n"/>
       <c r="N89" s="119" t="n"/>
       <c r="O89" s="119" t="n"/>
-      <c r="P89" s="146" t="n">
+      <c r="P89" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15823,7 +15819,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D90" s="146" t="n">
+      <c r="D90" s="119" t="n">
         <v>4269.55</v>
       </c>
       <c r="E90" s="119" t="n"/>
@@ -15837,7 +15833,7 @@
       <c r="M90" s="119" t="n"/>
       <c r="N90" s="119" t="n"/>
       <c r="O90" s="119" t="n"/>
-      <c r="P90" s="146" t="n">
+      <c r="P90" s="119" t="n">
         <v>4269.55</v>
       </c>
     </row>
@@ -15857,7 +15853,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D91" s="145" t="n">
+      <c r="D91" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E91" s="116" t="n"/>
@@ -15871,7 +15867,7 @@
       <c r="M91" s="116" t="n"/>
       <c r="N91" s="116" t="n"/>
       <c r="O91" s="116" t="n"/>
-      <c r="P91" s="145" t="n">
+      <c r="P91" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15891,7 +15887,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D92" s="146" t="n">
+      <c r="D92" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E92" s="119" t="n"/>
@@ -15905,7 +15901,7 @@
       <c r="M92" s="119" t="n"/>
       <c r="N92" s="119" t="n"/>
       <c r="O92" s="119" t="n"/>
-      <c r="P92" s="146" t="n">
+      <c r="P92" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15925,7 +15921,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D93" s="146" t="n">
+      <c r="D93" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E93" s="119" t="n"/>
@@ -15939,7 +15935,7 @@
       <c r="M93" s="119" t="n"/>
       <c r="N93" s="119" t="n"/>
       <c r="O93" s="119" t="n"/>
-      <c r="P93" s="146" t="n">
+      <c r="P93" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15959,7 +15955,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D94" s="145" t="n">
+      <c r="D94" s="116" t="n">
         <v>10317.24</v>
       </c>
       <c r="E94" s="116" t="n"/>
@@ -15973,7 +15969,7 @@
       <c r="M94" s="116" t="n"/>
       <c r="N94" s="116" t="n"/>
       <c r="O94" s="116" t="n"/>
-      <c r="P94" s="145" t="n">
+      <c r="P94" s="116" t="n">
         <v>10317.24</v>
       </c>
     </row>
@@ -15993,7 +15989,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D95" s="146" t="n">
+      <c r="D95" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E95" s="119" t="n"/>
@@ -16007,7 +16003,7 @@
       <c r="M95" s="119" t="n"/>
       <c r="N95" s="119" t="n"/>
       <c r="O95" s="119" t="n"/>
-      <c r="P95" s="146" t="n">
+      <c r="P95" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16027,7 +16023,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D96" s="146" t="n">
+      <c r="D96" s="119" t="n">
         <v>10317.24</v>
       </c>
       <c r="E96" s="119" t="n"/>
@@ -16041,7 +16037,7 @@
       <c r="M96" s="119" t="n"/>
       <c r="N96" s="119" t="n"/>
       <c r="O96" s="119" t="n"/>
-      <c r="P96" s="146" t="n">
+      <c r="P96" s="119" t="n">
         <v>10317.24</v>
       </c>
     </row>
@@ -16061,7 +16057,7 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D97" s="145" t="n">
+      <c r="D97" s="116" t="n">
         <v>0</v>
       </c>
       <c r="E97" s="116" t="n"/>
@@ -16075,7 +16071,7 @@
       <c r="M97" s="116" t="n"/>
       <c r="N97" s="116" t="n"/>
       <c r="O97" s="116" t="n"/>
-      <c r="P97" s="145" t="n">
+      <c r="P97" s="116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16095,7 +16091,7 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D98" s="146" t="n">
+      <c r="D98" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E98" s="119" t="n"/>
@@ -16109,7 +16105,7 @@
       <c r="M98" s="119" t="n"/>
       <c r="N98" s="119" t="n"/>
       <c r="O98" s="119" t="n"/>
-      <c r="P98" s="146" t="n">
+      <c r="P98" s="119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16129,7 +16125,7 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D99" s="146" t="n">
+      <c r="D99" s="119" t="n">
         <v>0</v>
       </c>
       <c r="E99" s="119" t="n"/>
@@ -16143,55 +16139,55 @@
       <c r="M99" s="119" t="n"/>
       <c r="N99" s="119" t="n"/>
       <c r="O99" s="119" t="n"/>
-      <c r="P99" s="146" t="n">
+      <c r="P99" s="119" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="100" ht="35.25" customHeight="1" s="134">
       <c r="A100" s="123" t="inlineStr">
         <is>
-          <t>total meses:</t>
+          <t>TOTAL MESES:</t>
         </is>
       </c>
       <c r="B100" s="138" t="n"/>
       <c r="C100" s="136" t="n"/>
-      <c r="D100" s="148" t="n">
+      <c r="D100" s="121" t="n">
         <v>72870.70000000001</v>
       </c>
-      <c r="E100" s="148" t="n">
+      <c r="E100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="F100" s="148" t="n">
+      <c r="F100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="G100" s="148" t="n">
+      <c r="G100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="H100" s="148" t="n">
+      <c r="H100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="I100" s="148" t="n">
+      <c r="I100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="J100" s="148" t="n">
+      <c r="J100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="K100" s="148" t="n">
+      <c r="K100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="L100" s="148" t="n">
+      <c r="L100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="M100" s="148" t="n">
+      <c r="M100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="N100" s="148" t="n">
+      <c r="N100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="O100" s="148" t="n">
+      <c r="O100" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="P100" s="148" t="n">
+      <c r="P100" s="121" t="n">
         <v>72870.70000000001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização do app.py para leitura de word
</commit_message>
<xml_diff>
--- a/exit/Meta49_preenchido.xlsx
+++ b/exit/Meta49_preenchido.xlsx
@@ -12895,10 +12895,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D4" s="116" t="n">
+      <c r="D4" s="116" t="n"/>
+      <c r="E4" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="116" t="n"/>
       <c r="F4" s="116" t="n"/>
       <c r="G4" s="116" t="n"/>
       <c r="H4" s="116" t="n"/>
@@ -12929,10 +12929,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D5" s="119" t="n">
+      <c r="D5" s="119" t="n"/>
+      <c r="E5" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="119" t="n"/>
       <c r="F5" s="119" t="n"/>
       <c r="G5" s="119" t="n"/>
       <c r="H5" s="119" t="n"/>
@@ -12963,10 +12963,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D6" s="119" t="n">
+      <c r="D6" s="119" t="n"/>
+      <c r="E6" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="119" t="n"/>
       <c r="F6" s="119" t="n"/>
       <c r="G6" s="119" t="n"/>
       <c r="H6" s="119" t="n"/>
@@ -12997,10 +12997,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D7" s="116" t="n">
+      <c r="D7" s="116" t="n"/>
+      <c r="E7" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="116" t="n"/>
       <c r="F7" s="116" t="n"/>
       <c r="G7" s="116" t="n"/>
       <c r="H7" s="116" t="n"/>
@@ -13031,10 +13031,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D8" s="119" t="n">
+      <c r="D8" s="119" t="n"/>
+      <c r="E8" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="119" t="n"/>
       <c r="F8" s="119" t="n"/>
       <c r="G8" s="119" t="n"/>
       <c r="H8" s="119" t="n"/>
@@ -13065,10 +13065,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D9" s="119" t="n">
+      <c r="D9" s="119" t="n"/>
+      <c r="E9" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="119" t="n"/>
       <c r="F9" s="119" t="n"/>
       <c r="G9" s="119" t="n"/>
       <c r="H9" s="119" t="n"/>
@@ -13099,10 +13099,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D10" s="116" t="n">
+      <c r="D10" s="116" t="n"/>
+      <c r="E10" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="116" t="n"/>
       <c r="F10" s="116" t="n"/>
       <c r="G10" s="116" t="n"/>
       <c r="H10" s="116" t="n"/>
@@ -13133,10 +13133,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D11" s="119" t="n">
+      <c r="D11" s="119" t="n"/>
+      <c r="E11" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="119" t="n"/>
       <c r="F11" s="119" t="n"/>
       <c r="G11" s="119" t="n"/>
       <c r="H11" s="119" t="n"/>
@@ -13167,10 +13167,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D12" s="119" t="n">
+      <c r="D12" s="119" t="n"/>
+      <c r="E12" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="119" t="n"/>
       <c r="F12" s="119" t="n"/>
       <c r="G12" s="119" t="n"/>
       <c r="H12" s="119" t="n"/>
@@ -13201,10 +13201,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D13" s="116" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="116" t="n"/>
+      <c r="D13" s="116" t="n"/>
+      <c r="E13" s="116" t="n">
+        <v>25308</v>
+      </c>
       <c r="F13" s="116" t="n"/>
       <c r="G13" s="116" t="n"/>
       <c r="H13" s="116" t="n"/>
@@ -13216,7 +13216,7 @@
       <c r="N13" s="116" t="n"/>
       <c r="O13" s="116" t="n"/>
       <c r="P13" s="116" t="n">
-        <v>0</v>
+        <v>25308</v>
       </c>
     </row>
     <row r="14" ht="35.25" customHeight="1" s="134">
@@ -13235,10 +13235,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D14" s="119" t="n">
+      <c r="D14" s="119" t="n"/>
+      <c r="E14" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="119" t="n"/>
       <c r="F14" s="119" t="n"/>
       <c r="G14" s="119" t="n"/>
       <c r="H14" s="119" t="n"/>
@@ -13269,10 +13269,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D15" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="119" t="n"/>
+      <c r="D15" s="119" t="n"/>
+      <c r="E15" s="119" t="n">
+        <v>25308</v>
+      </c>
       <c r="F15" s="119" t="n"/>
       <c r="G15" s="119" t="n"/>
       <c r="H15" s="119" t="n"/>
@@ -13284,7 +13284,7 @@
       <c r="N15" s="119" t="n"/>
       <c r="O15" s="119" t="n"/>
       <c r="P15" s="119" t="n">
-        <v>0</v>
+        <v>25308</v>
       </c>
     </row>
     <row r="16" ht="35.25" customHeight="1" s="134">
@@ -13303,10 +13303,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D16" s="116" t="n">
+      <c r="D16" s="116" t="n"/>
+      <c r="E16" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="116" t="n"/>
       <c r="F16" s="116" t="n"/>
       <c r="G16" s="116" t="n"/>
       <c r="H16" s="116" t="n"/>
@@ -13337,10 +13337,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D17" s="119" t="n">
+      <c r="D17" s="119" t="n"/>
+      <c r="E17" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="119" t="n"/>
       <c r="F17" s="119" t="n"/>
       <c r="G17" s="119" t="n"/>
       <c r="H17" s="119" t="n"/>
@@ -13371,10 +13371,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D18" s="119" t="n">
+      <c r="D18" s="119" t="n"/>
+      <c r="E18" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="119" t="n"/>
       <c r="F18" s="119" t="n"/>
       <c r="G18" s="119" t="n"/>
       <c r="H18" s="119" t="n"/>
@@ -13405,10 +13405,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D19" s="116" t="n">
+      <c r="D19" s="116" t="n"/>
+      <c r="E19" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="116" t="n"/>
       <c r="F19" s="116" t="n"/>
       <c r="G19" s="116" t="n"/>
       <c r="H19" s="116" t="n"/>
@@ -13439,10 +13439,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D20" s="119" t="n">
+      <c r="D20" s="119" t="n"/>
+      <c r="E20" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="119" t="n"/>
       <c r="F20" s="119" t="n"/>
       <c r="G20" s="119" t="n"/>
       <c r="H20" s="119" t="n"/>
@@ -13473,10 +13473,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D21" s="119" t="n">
+      <c r="D21" s="119" t="n"/>
+      <c r="E21" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="119" t="n"/>
       <c r="F21" s="119" t="n"/>
       <c r="G21" s="119" t="n"/>
       <c r="H21" s="119" t="n"/>
@@ -13507,10 +13507,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D22" s="116" t="n">
-        <v>17631</v>
-      </c>
-      <c r="E22" s="116" t="n"/>
+      <c r="D22" s="116" t="n"/>
+      <c r="E22" s="116" t="n">
+        <v>7013.4</v>
+      </c>
       <c r="F22" s="116" t="n"/>
       <c r="G22" s="116" t="n"/>
       <c r="H22" s="116" t="n"/>
@@ -13522,7 +13522,7 @@
       <c r="N22" s="116" t="n"/>
       <c r="O22" s="116" t="n"/>
       <c r="P22" s="116" t="n">
-        <v>17631</v>
+        <v>7013.4</v>
       </c>
     </row>
     <row r="23" ht="35.25" customHeight="1" s="134">
@@ -13541,10 +13541,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D23" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="119" t="n"/>
+      <c r="D23" s="119" t="n"/>
+      <c r="E23" s="119" t="n">
+        <v>3143.4</v>
+      </c>
       <c r="F23" s="119" t="n"/>
       <c r="G23" s="119" t="n"/>
       <c r="H23" s="119" t="n"/>
@@ -13556,7 +13556,7 @@
       <c r="N23" s="119" t="n"/>
       <c r="O23" s="119" t="n"/>
       <c r="P23" s="119" t="n">
-        <v>0</v>
+        <v>3143.4</v>
       </c>
     </row>
     <row r="24" ht="35.25" customHeight="1" s="134">
@@ -13575,10 +13575,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D24" s="119" t="n">
-        <v>17631</v>
-      </c>
-      <c r="E24" s="119" t="n"/>
+      <c r="D24" s="119" t="n"/>
+      <c r="E24" s="119" t="n">
+        <v>3870</v>
+      </c>
       <c r="F24" s="119" t="n"/>
       <c r="G24" s="119" t="n"/>
       <c r="H24" s="119" t="n"/>
@@ -13590,7 +13590,7 @@
       <c r="N24" s="119" t="n"/>
       <c r="O24" s="119" t="n"/>
       <c r="P24" s="119" t="n">
-        <v>17631</v>
+        <v>3870</v>
       </c>
     </row>
     <row r="25" ht="35.25" customHeight="1" s="134">
@@ -13609,10 +13609,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D25" s="116" t="n">
+      <c r="D25" s="116" t="n"/>
+      <c r="E25" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="116" t="n"/>
       <c r="F25" s="116" t="n"/>
       <c r="G25" s="116" t="n"/>
       <c r="H25" s="116" t="n"/>
@@ -13643,10 +13643,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D26" s="119" t="n">
+      <c r="D26" s="119" t="n"/>
+      <c r="E26" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="119" t="n"/>
       <c r="F26" s="119" t="n"/>
       <c r="G26" s="119" t="n"/>
       <c r="H26" s="119" t="n"/>
@@ -13677,10 +13677,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D27" s="119" t="n">
+      <c r="D27" s="119" t="n"/>
+      <c r="E27" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E27" s="119" t="n"/>
       <c r="F27" s="119" t="n"/>
       <c r="G27" s="119" t="n"/>
       <c r="H27" s="119" t="n"/>
@@ -13711,10 +13711,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D28" s="116" t="n">
-        <v>2840.1</v>
-      </c>
-      <c r="E28" s="116" t="n"/>
+      <c r="D28" s="116" t="n"/>
+      <c r="E28" s="116" t="n">
+        <v>27588.24</v>
+      </c>
       <c r="F28" s="116" t="n"/>
       <c r="G28" s="116" t="n"/>
       <c r="H28" s="116" t="n"/>
@@ -13726,7 +13726,7 @@
       <c r="N28" s="116" t="n"/>
       <c r="O28" s="116" t="n"/>
       <c r="P28" s="116" t="n">
-        <v>2840.1</v>
+        <v>27588.24</v>
       </c>
     </row>
     <row r="29" ht="35.25" customHeight="1" s="134">
@@ -13745,10 +13745,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D29" s="119" t="n">
-        <v>2840.1</v>
-      </c>
-      <c r="E29" s="119" t="n"/>
+      <c r="D29" s="119" t="n"/>
+      <c r="E29" s="119" t="n">
+        <v>27588.24</v>
+      </c>
       <c r="F29" s="119" t="n"/>
       <c r="G29" s="119" t="n"/>
       <c r="H29" s="119" t="n"/>
@@ -13760,7 +13760,7 @@
       <c r="N29" s="119" t="n"/>
       <c r="O29" s="119" t="n"/>
       <c r="P29" s="119" t="n">
-        <v>2840.1</v>
+        <v>27588.24</v>
       </c>
     </row>
     <row r="30" ht="35.25" customHeight="1" s="134">
@@ -13779,10 +13779,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D30" s="119" t="n">
+      <c r="D30" s="119" t="n"/>
+      <c r="E30" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="119" t="n"/>
       <c r="F30" s="119" t="n"/>
       <c r="G30" s="119" t="n"/>
       <c r="H30" s="119" t="n"/>
@@ -13813,10 +13813,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D31" s="116" t="n">
+      <c r="D31" s="116" t="n"/>
+      <c r="E31" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E31" s="116" t="n"/>
       <c r="F31" s="116" t="n"/>
       <c r="G31" s="116" t="n"/>
       <c r="H31" s="116" t="n"/>
@@ -13847,10 +13847,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D32" s="119" t="n">
+      <c r="D32" s="119" t="n"/>
+      <c r="E32" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="119" t="n"/>
       <c r="F32" s="119" t="n"/>
       <c r="G32" s="119" t="n"/>
       <c r="H32" s="119" t="n"/>
@@ -13881,10 +13881,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D33" s="119" t="n">
+      <c r="D33" s="119" t="n"/>
+      <c r="E33" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E33" s="119" t="n"/>
       <c r="F33" s="119" t="n"/>
       <c r="G33" s="119" t="n"/>
       <c r="H33" s="119" t="n"/>
@@ -13915,10 +13915,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D34" s="116" t="n">
+      <c r="D34" s="116" t="n"/>
+      <c r="E34" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="116" t="n"/>
       <c r="F34" s="116" t="n"/>
       <c r="G34" s="116" t="n"/>
       <c r="H34" s="116" t="n"/>
@@ -13949,10 +13949,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D35" s="119" t="n">
+      <c r="D35" s="119" t="n"/>
+      <c r="E35" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="119" t="n"/>
       <c r="F35" s="119" t="n"/>
       <c r="G35" s="119" t="n"/>
       <c r="H35" s="119" t="n"/>
@@ -13983,10 +13983,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D36" s="119" t="n">
+      <c r="D36" s="119" t="n"/>
+      <c r="E36" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="119" t="n"/>
       <c r="F36" s="119" t="n"/>
       <c r="G36" s="119" t="n"/>
       <c r="H36" s="119" t="n"/>
@@ -14017,10 +14017,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D37" s="116" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="116" t="n"/>
+      <c r="D37" s="116" t="n"/>
+      <c r="E37" s="116" t="n">
+        <v>3760</v>
+      </c>
       <c r="F37" s="116" t="n"/>
       <c r="G37" s="116" t="n"/>
       <c r="H37" s="116" t="n"/>
@@ -14032,7 +14032,7 @@
       <c r="N37" s="116" t="n"/>
       <c r="O37" s="116" t="n"/>
       <c r="P37" s="116" t="n">
-        <v>0</v>
+        <v>3760</v>
       </c>
     </row>
     <row r="38" ht="35.25" customHeight="1" s="134">
@@ -14051,10 +14051,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D38" s="119" t="n">
+      <c r="D38" s="119" t="n"/>
+      <c r="E38" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E38" s="119" t="n"/>
       <c r="F38" s="119" t="n"/>
       <c r="G38" s="119" t="n"/>
       <c r="H38" s="119" t="n"/>
@@ -14085,10 +14085,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D39" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="119" t="n"/>
+      <c r="D39" s="119" t="n"/>
+      <c r="E39" s="119" t="n">
+        <v>3760</v>
+      </c>
       <c r="F39" s="119" t="n"/>
       <c r="G39" s="119" t="n"/>
       <c r="H39" s="119" t="n"/>
@@ -14100,7 +14100,7 @@
       <c r="N39" s="119" t="n"/>
       <c r="O39" s="119" t="n"/>
       <c r="P39" s="119" t="n">
-        <v>0</v>
+        <v>3760</v>
       </c>
     </row>
     <row r="40" ht="35.25" customHeight="1" s="134">
@@ -14119,10 +14119,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D40" s="116" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="116" t="n"/>
+      <c r="D40" s="116" t="n"/>
+      <c r="E40" s="116" t="n">
+        <v>3486.51</v>
+      </c>
       <c r="F40" s="116" t="n"/>
       <c r="G40" s="116" t="n"/>
       <c r="H40" s="116" t="n"/>
@@ -14134,7 +14134,7 @@
       <c r="N40" s="116" t="n"/>
       <c r="O40" s="116" t="n"/>
       <c r="P40" s="116" t="n">
-        <v>0</v>
+        <v>3486.51</v>
       </c>
     </row>
     <row r="41" ht="35.25" customHeight="1" s="134">
@@ -14153,10 +14153,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D41" s="119" t="n">
+      <c r="D41" s="119" t="n"/>
+      <c r="E41" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E41" s="119" t="n"/>
       <c r="F41" s="119" t="n"/>
       <c r="G41" s="119" t="n"/>
       <c r="H41" s="119" t="n"/>
@@ -14187,10 +14187,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D42" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" s="119" t="n"/>
+      <c r="D42" s="119" t="n"/>
+      <c r="E42" s="119" t="n">
+        <v>3486.51</v>
+      </c>
       <c r="F42" s="119" t="n"/>
       <c r="G42" s="119" t="n"/>
       <c r="H42" s="119" t="n"/>
@@ -14202,7 +14202,7 @@
       <c r="N42" s="119" t="n"/>
       <c r="O42" s="119" t="n"/>
       <c r="P42" s="119" t="n">
-        <v>0</v>
+        <v>3486.51</v>
       </c>
     </row>
     <row r="43" ht="35.25" customHeight="1" s="134">
@@ -14221,10 +14221,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D43" s="116" t="n">
+      <c r="D43" s="116" t="n"/>
+      <c r="E43" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E43" s="116" t="n"/>
       <c r="F43" s="116" t="n"/>
       <c r="G43" s="116" t="n"/>
       <c r="H43" s="116" t="n"/>
@@ -14255,10 +14255,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D44" s="119" t="n">
+      <c r="D44" s="119" t="n"/>
+      <c r="E44" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E44" s="119" t="n"/>
       <c r="F44" s="119" t="n"/>
       <c r="G44" s="119" t="n"/>
       <c r="H44" s="119" t="n"/>
@@ -14289,10 +14289,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D45" s="119" t="n">
+      <c r="D45" s="119" t="n"/>
+      <c r="E45" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E45" s="119" t="n"/>
       <c r="F45" s="119" t="n"/>
       <c r="G45" s="119" t="n"/>
       <c r="H45" s="119" t="n"/>
@@ -14323,10 +14323,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D46" s="116" t="n">
-        <v>16322.7</v>
-      </c>
-      <c r="E46" s="116" t="n"/>
+      <c r="D46" s="116" t="n"/>
+      <c r="E46" s="116" t="n">
+        <v>24149.35</v>
+      </c>
       <c r="F46" s="116" t="n"/>
       <c r="G46" s="116" t="n"/>
       <c r="H46" s="116" t="n"/>
@@ -14338,7 +14338,7 @@
       <c r="N46" s="116" t="n"/>
       <c r="O46" s="116" t="n"/>
       <c r="P46" s="116" t="n">
-        <v>16322.7</v>
+        <v>24149.35</v>
       </c>
     </row>
     <row r="47" ht="35.25" customHeight="1" s="134">
@@ -14357,10 +14357,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D47" s="119" t="n">
-        <v>2897.7</v>
-      </c>
-      <c r="E47" s="119" t="n"/>
+      <c r="D47" s="119" t="n"/>
+      <c r="E47" s="119" t="n">
+        <v>5210.35</v>
+      </c>
       <c r="F47" s="119" t="n"/>
       <c r="G47" s="119" t="n"/>
       <c r="H47" s="119" t="n"/>
@@ -14372,7 +14372,7 @@
       <c r="N47" s="119" t="n"/>
       <c r="O47" s="119" t="n"/>
       <c r="P47" s="119" t="n">
-        <v>2897.7</v>
+        <v>5210.35</v>
       </c>
     </row>
     <row r="48" ht="35.25" customHeight="1" s="134">
@@ -14391,10 +14391,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D48" s="119" t="n">
-        <v>13425</v>
-      </c>
-      <c r="E48" s="119" t="n"/>
+      <c r="D48" s="119" t="n"/>
+      <c r="E48" s="119" t="n">
+        <v>18939</v>
+      </c>
       <c r="F48" s="119" t="n"/>
       <c r="G48" s="119" t="n"/>
       <c r="H48" s="119" t="n"/>
@@ -14406,7 +14406,7 @@
       <c r="N48" s="119" t="n"/>
       <c r="O48" s="119" t="n"/>
       <c r="P48" s="119" t="n">
-        <v>13425</v>
+        <v>18939</v>
       </c>
     </row>
     <row r="49" ht="35.25" customHeight="1" s="134">
@@ -14425,10 +14425,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D49" s="116" t="n">
+      <c r="D49" s="116" t="n"/>
+      <c r="E49" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E49" s="116" t="n"/>
       <c r="F49" s="116" t="n"/>
       <c r="G49" s="116" t="n"/>
       <c r="H49" s="116" t="n"/>
@@ -14459,10 +14459,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D50" s="119" t="n">
+      <c r="D50" s="119" t="n"/>
+      <c r="E50" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E50" s="119" t="n"/>
       <c r="F50" s="119" t="n"/>
       <c r="G50" s="119" t="n"/>
       <c r="H50" s="119" t="n"/>
@@ -14493,10 +14493,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D51" s="119" t="n">
+      <c r="D51" s="119" t="n"/>
+      <c r="E51" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E51" s="119" t="n"/>
       <c r="F51" s="119" t="n"/>
       <c r="G51" s="119" t="n"/>
       <c r="H51" s="119" t="n"/>
@@ -14527,10 +14527,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D52" s="116" t="n">
+      <c r="D52" s="116" t="n"/>
+      <c r="E52" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E52" s="116" t="n"/>
       <c r="F52" s="116" t="n"/>
       <c r="G52" s="116" t="n"/>
       <c r="H52" s="116" t="n"/>
@@ -14561,10 +14561,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D53" s="119" t="n">
+      <c r="D53" s="119" t="n"/>
+      <c r="E53" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E53" s="119" t="n"/>
       <c r="F53" s="119" t="n"/>
       <c r="G53" s="119" t="n"/>
       <c r="H53" s="119" t="n"/>
@@ -14595,10 +14595,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D54" s="119" t="n">
+      <c r="D54" s="119" t="n"/>
+      <c r="E54" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E54" s="119" t="n"/>
       <c r="F54" s="119" t="n"/>
       <c r="G54" s="119" t="n"/>
       <c r="H54" s="119" t="n"/>
@@ -14629,10 +14629,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D55" s="116" t="n">
-        <v>1066</v>
-      </c>
-      <c r="E55" s="116" t="n"/>
+      <c r="D55" s="116" t="n"/>
+      <c r="E55" s="116" t="n">
+        <v>0</v>
+      </c>
       <c r="F55" s="116" t="n"/>
       <c r="G55" s="116" t="n"/>
       <c r="H55" s="116" t="n"/>
@@ -14644,7 +14644,7 @@
       <c r="N55" s="116" t="n"/>
       <c r="O55" s="116" t="n"/>
       <c r="P55" s="116" t="n">
-        <v>1066</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" ht="35.25" customHeight="1" s="134">
@@ -14663,10 +14663,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D56" s="119" t="n">
-        <v>1066</v>
-      </c>
-      <c r="E56" s="119" t="n"/>
+      <c r="D56" s="119" t="n"/>
+      <c r="E56" s="119" t="n">
+        <v>0</v>
+      </c>
       <c r="F56" s="119" t="n"/>
       <c r="G56" s="119" t="n"/>
       <c r="H56" s="119" t="n"/>
@@ -14678,7 +14678,7 @@
       <c r="N56" s="119" t="n"/>
       <c r="O56" s="119" t="n"/>
       <c r="P56" s="119" t="n">
-        <v>1066</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" ht="35.25" customHeight="1" s="134">
@@ -14697,10 +14697,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D57" s="119" t="n">
+      <c r="D57" s="119" t="n"/>
+      <c r="E57" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E57" s="119" t="n"/>
       <c r="F57" s="119" t="n"/>
       <c r="G57" s="119" t="n"/>
       <c r="H57" s="119" t="n"/>
@@ -14731,10 +14731,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D58" s="116" t="n">
+      <c r="D58" s="116" t="n"/>
+      <c r="E58" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E58" s="116" t="n"/>
       <c r="F58" s="116" t="n"/>
       <c r="G58" s="116" t="n"/>
       <c r="H58" s="116" t="n"/>
@@ -14765,10 +14765,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D59" s="119" t="n">
+      <c r="D59" s="119" t="n"/>
+      <c r="E59" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E59" s="119" t="n"/>
       <c r="F59" s="119" t="n"/>
       <c r="G59" s="119" t="n"/>
       <c r="H59" s="119" t="n"/>
@@ -14799,10 +14799,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D60" s="119" t="n">
+      <c r="D60" s="119" t="n"/>
+      <c r="E60" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E60" s="119" t="n"/>
       <c r="F60" s="119" t="n"/>
       <c r="G60" s="119" t="n"/>
       <c r="H60" s="119" t="n"/>
@@ -14833,10 +14833,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D61" s="116" t="n">
-        <v>7912.81</v>
-      </c>
-      <c r="E61" s="116" t="n"/>
+      <c r="D61" s="116" t="n"/>
+      <c r="E61" s="116" t="n">
+        <v>20737.16</v>
+      </c>
       <c r="F61" s="116" t="n"/>
       <c r="G61" s="116" t="n"/>
       <c r="H61" s="116" t="n"/>
@@ -14848,7 +14848,7 @@
       <c r="N61" s="116" t="n"/>
       <c r="O61" s="116" t="n"/>
       <c r="P61" s="116" t="n">
-        <v>7912.81</v>
+        <v>20737.16</v>
       </c>
     </row>
     <row r="62" ht="35.25" customHeight="1" s="134">
@@ -14867,10 +14867,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D62" s="119" t="n">
+      <c r="D62" s="119" t="n"/>
+      <c r="E62" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E62" s="119" t="n"/>
       <c r="F62" s="119" t="n"/>
       <c r="G62" s="119" t="n"/>
       <c r="H62" s="119" t="n"/>
@@ -14901,10 +14901,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D63" s="119" t="n">
-        <v>7912.81</v>
-      </c>
-      <c r="E63" s="119" t="n"/>
+      <c r="D63" s="119" t="n"/>
+      <c r="E63" s="119" t="n">
+        <v>20737.16</v>
+      </c>
       <c r="F63" s="119" t="n"/>
       <c r="G63" s="119" t="n"/>
       <c r="H63" s="119" t="n"/>
@@ -14916,7 +14916,7 @@
       <c r="N63" s="119" t="n"/>
       <c r="O63" s="119" t="n"/>
       <c r="P63" s="119" t="n">
-        <v>7912.81</v>
+        <v>20737.16</v>
       </c>
     </row>
     <row r="64" ht="35.25" customHeight="1" s="134">
@@ -14935,10 +14935,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D64" s="116" t="n">
+      <c r="D64" s="116" t="n"/>
+      <c r="E64" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E64" s="116" t="n"/>
       <c r="F64" s="116" t="n"/>
       <c r="G64" s="116" t="n"/>
       <c r="H64" s="116" t="n"/>
@@ -14969,10 +14969,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D65" s="119" t="n">
+      <c r="D65" s="119" t="n"/>
+      <c r="E65" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E65" s="119" t="n"/>
       <c r="F65" s="119" t="n"/>
       <c r="G65" s="119" t="n"/>
       <c r="H65" s="119" t="n"/>
@@ -15003,10 +15003,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D66" s="119" t="n">
+      <c r="D66" s="119" t="n"/>
+      <c r="E66" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E66" s="119" t="n"/>
       <c r="F66" s="119" t="n"/>
       <c r="G66" s="119" t="n"/>
       <c r="H66" s="119" t="n"/>
@@ -15037,10 +15037,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D67" s="116" t="n">
-        <v>0</v>
-      </c>
-      <c r="E67" s="116" t="n"/>
+      <c r="D67" s="116" t="n"/>
+      <c r="E67" s="116" t="n">
+        <v>3030.71</v>
+      </c>
       <c r="F67" s="116" t="n"/>
       <c r="G67" s="116" t="n"/>
       <c r="H67" s="116" t="n"/>
@@ -15052,7 +15052,7 @@
       <c r="N67" s="116" t="n"/>
       <c r="O67" s="116" t="n"/>
       <c r="P67" s="116" t="n">
-        <v>0</v>
+        <v>3030.71</v>
       </c>
     </row>
     <row r="68" ht="35.25" customHeight="1" s="134">
@@ -15071,10 +15071,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D68" s="119" t="n">
+      <c r="D68" s="119" t="n"/>
+      <c r="E68" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E68" s="119" t="n"/>
       <c r="F68" s="119" t="n"/>
       <c r="G68" s="119" t="n"/>
       <c r="H68" s="119" t="n"/>
@@ -15105,10 +15105,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D69" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="119" t="n"/>
+      <c r="D69" s="119" t="n"/>
+      <c r="E69" s="119" t="n">
+        <v>3030.71</v>
+      </c>
       <c r="F69" s="119" t="n"/>
       <c r="G69" s="119" t="n"/>
       <c r="H69" s="119" t="n"/>
@@ -15120,7 +15120,7 @@
       <c r="N69" s="119" t="n"/>
       <c r="O69" s="119" t="n"/>
       <c r="P69" s="119" t="n">
-        <v>0</v>
+        <v>3030.71</v>
       </c>
     </row>
     <row r="70" ht="35.25" customHeight="1" s="134">
@@ -15139,10 +15139,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D70" s="116" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="116" t="n"/>
+      <c r="D70" s="116" t="n"/>
+      <c r="E70" s="116" t="n">
+        <v>2055</v>
+      </c>
       <c r="F70" s="116" t="n"/>
       <c r="G70" s="116" t="n"/>
       <c r="H70" s="116" t="n"/>
@@ -15154,7 +15154,7 @@
       <c r="N70" s="116" t="n"/>
       <c r="O70" s="116" t="n"/>
       <c r="P70" s="116" t="n">
-        <v>0</v>
+        <v>2055</v>
       </c>
     </row>
     <row r="71" ht="35.25" customHeight="1" s="134">
@@ -15173,10 +15173,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D71" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="E71" s="119" t="n"/>
+      <c r="D71" s="119" t="n"/>
+      <c r="E71" s="119" t="n">
+        <v>2055</v>
+      </c>
       <c r="F71" s="119" t="n"/>
       <c r="G71" s="119" t="n"/>
       <c r="H71" s="119" t="n"/>
@@ -15188,7 +15188,7 @@
       <c r="N71" s="119" t="n"/>
       <c r="O71" s="119" t="n"/>
       <c r="P71" s="119" t="n">
-        <v>0</v>
+        <v>2055</v>
       </c>
     </row>
     <row r="72" ht="35.25" customHeight="1" s="134">
@@ -15207,10 +15207,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D72" s="119" t="n">
+      <c r="D72" s="119" t="n"/>
+      <c r="E72" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E72" s="119" t="n"/>
       <c r="F72" s="119" t="n"/>
       <c r="G72" s="119" t="n"/>
       <c r="H72" s="119" t="n"/>
@@ -15241,10 +15241,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D73" s="116" t="n">
-        <v>3041.3</v>
-      </c>
-      <c r="E73" s="116" t="n"/>
+      <c r="D73" s="116" t="n"/>
+      <c r="E73" s="116" t="n">
+        <v>8126.36</v>
+      </c>
       <c r="F73" s="116" t="n"/>
       <c r="G73" s="116" t="n"/>
       <c r="H73" s="116" t="n"/>
@@ -15256,7 +15256,7 @@
       <c r="N73" s="116" t="n"/>
       <c r="O73" s="116" t="n"/>
       <c r="P73" s="116" t="n">
-        <v>3041.3</v>
+        <v>8126.36</v>
       </c>
     </row>
     <row r="74" ht="35.25" customHeight="1" s="134">
@@ -15275,10 +15275,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D74" s="119" t="n">
-        <v>3041.3</v>
-      </c>
-      <c r="E74" s="119" t="n"/>
+      <c r="D74" s="119" t="n"/>
+      <c r="E74" s="119" t="n">
+        <v>8126.36</v>
+      </c>
       <c r="F74" s="119" t="n"/>
       <c r="G74" s="119" t="n"/>
       <c r="H74" s="119" t="n"/>
@@ -15290,7 +15290,7 @@
       <c r="N74" s="119" t="n"/>
       <c r="O74" s="119" t="n"/>
       <c r="P74" s="119" t="n">
-        <v>3041.3</v>
+        <v>8126.36</v>
       </c>
     </row>
     <row r="75" ht="35.25" customHeight="1" s="134">
@@ -15309,10 +15309,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D75" s="119" t="n">
+      <c r="D75" s="119" t="n"/>
+      <c r="E75" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E75" s="119" t="n"/>
       <c r="F75" s="119" t="n"/>
       <c r="G75" s="119" t="n"/>
       <c r="H75" s="119" t="n"/>
@@ -15343,10 +15343,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D76" s="116" t="n">
+      <c r="D76" s="116" t="n"/>
+      <c r="E76" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E76" s="116" t="n"/>
       <c r="F76" s="116" t="n"/>
       <c r="G76" s="116" t="n"/>
       <c r="H76" s="116" t="n"/>
@@ -15377,10 +15377,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D77" s="119" t="n">
+      <c r="D77" s="119" t="n"/>
+      <c r="E77" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E77" s="119" t="n"/>
       <c r="F77" s="119" t="n"/>
       <c r="G77" s="119" t="n"/>
       <c r="H77" s="119" t="n"/>
@@ -15411,10 +15411,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D78" s="119" t="n">
+      <c r="D78" s="119" t="n"/>
+      <c r="E78" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E78" s="119" t="n"/>
       <c r="F78" s="119" t="n"/>
       <c r="G78" s="119" t="n"/>
       <c r="H78" s="119" t="n"/>
@@ -15445,10 +15445,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D79" s="116" t="n">
+      <c r="D79" s="116" t="n"/>
+      <c r="E79" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E79" s="116" t="n"/>
       <c r="F79" s="116" t="n"/>
       <c r="G79" s="116" t="n"/>
       <c r="H79" s="116" t="n"/>
@@ -15479,10 +15479,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D80" s="119" t="n">
+      <c r="D80" s="119" t="n"/>
+      <c r="E80" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E80" s="119" t="n"/>
       <c r="F80" s="119" t="n"/>
       <c r="G80" s="119" t="n"/>
       <c r="H80" s="119" t="n"/>
@@ -15513,10 +15513,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D81" s="119" t="n">
+      <c r="D81" s="119" t="n"/>
+      <c r="E81" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E81" s="119" t="n"/>
       <c r="F81" s="119" t="n"/>
       <c r="G81" s="119" t="n"/>
       <c r="H81" s="119" t="n"/>
@@ -15547,10 +15547,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D82" s="116" t="n">
-        <v>2546</v>
-      </c>
-      <c r="E82" s="116" t="n"/>
+      <c r="D82" s="116" t="n"/>
+      <c r="E82" s="116" t="n">
+        <v>8195</v>
+      </c>
       <c r="F82" s="116" t="n"/>
       <c r="G82" s="116" t="n"/>
       <c r="H82" s="116" t="n"/>
@@ -15562,7 +15562,7 @@
       <c r="N82" s="116" t="n"/>
       <c r="O82" s="116" t="n"/>
       <c r="P82" s="116" t="n">
-        <v>2546</v>
+        <v>8195</v>
       </c>
     </row>
     <row r="83" ht="35.25" customHeight="1" s="134">
@@ -15581,10 +15581,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D83" s="119" t="n">
+      <c r="D83" s="119" t="n"/>
+      <c r="E83" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E83" s="119" t="n"/>
       <c r="F83" s="119" t="n"/>
       <c r="G83" s="119" t="n"/>
       <c r="H83" s="119" t="n"/>
@@ -15615,10 +15615,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D84" s="119" t="n">
-        <v>2546</v>
-      </c>
-      <c r="E84" s="119" t="n"/>
+      <c r="D84" s="119" t="n"/>
+      <c r="E84" s="119" t="n">
+        <v>8195</v>
+      </c>
       <c r="F84" s="119" t="n"/>
       <c r="G84" s="119" t="n"/>
       <c r="H84" s="119" t="n"/>
@@ -15630,7 +15630,7 @@
       <c r="N84" s="119" t="n"/>
       <c r="O84" s="119" t="n"/>
       <c r="P84" s="119" t="n">
-        <v>2546</v>
+        <v>8195</v>
       </c>
     </row>
     <row r="85" ht="35.25" customHeight="1" s="134">
@@ -15649,10 +15649,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D85" s="116" t="n">
-        <v>6924</v>
-      </c>
-      <c r="E85" s="116" t="n"/>
+      <c r="D85" s="116" t="n"/>
+      <c r="E85" s="116" t="n">
+        <v>0</v>
+      </c>
       <c r="F85" s="116" t="n"/>
       <c r="G85" s="116" t="n"/>
       <c r="H85" s="116" t="n"/>
@@ -15664,7 +15664,7 @@
       <c r="N85" s="116" t="n"/>
       <c r="O85" s="116" t="n"/>
       <c r="P85" s="116" t="n">
-        <v>6924</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" ht="35.25" customHeight="1" s="134">
@@ -15683,10 +15683,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D86" s="119" t="n">
+      <c r="D86" s="119" t="n"/>
+      <c r="E86" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E86" s="119" t="n"/>
       <c r="F86" s="119" t="n"/>
       <c r="G86" s="119" t="n"/>
       <c r="H86" s="119" t="n"/>
@@ -15717,10 +15717,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D87" s="119" t="n">
-        <v>6924</v>
-      </c>
-      <c r="E87" s="119" t="n"/>
+      <c r="D87" s="119" t="n"/>
+      <c r="E87" s="119" t="n">
+        <v>0</v>
+      </c>
       <c r="F87" s="119" t="n"/>
       <c r="G87" s="119" t="n"/>
       <c r="H87" s="119" t="n"/>
@@ -15732,7 +15732,7 @@
       <c r="N87" s="119" t="n"/>
       <c r="O87" s="119" t="n"/>
       <c r="P87" s="119" t="n">
-        <v>6924</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" ht="35.25" customHeight="1" s="134">
@@ -15751,10 +15751,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D88" s="116" t="n">
-        <v>4269.55</v>
-      </c>
-      <c r="E88" s="116" t="n"/>
+      <c r="D88" s="116" t="n"/>
+      <c r="E88" s="116" t="n">
+        <v>0</v>
+      </c>
       <c r="F88" s="116" t="n"/>
       <c r="G88" s="116" t="n"/>
       <c r="H88" s="116" t="n"/>
@@ -15766,7 +15766,7 @@
       <c r="N88" s="116" t="n"/>
       <c r="O88" s="116" t="n"/>
       <c r="P88" s="116" t="n">
-        <v>4269.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" ht="35.25" customHeight="1" s="134">
@@ -15785,10 +15785,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D89" s="119" t="n">
+      <c r="D89" s="119" t="n"/>
+      <c r="E89" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E89" s="119" t="n"/>
       <c r="F89" s="119" t="n"/>
       <c r="G89" s="119" t="n"/>
       <c r="H89" s="119" t="n"/>
@@ -15819,10 +15819,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D90" s="119" t="n">
-        <v>4269.55</v>
-      </c>
-      <c r="E90" s="119" t="n"/>
+      <c r="D90" s="119" t="n"/>
+      <c r="E90" s="119" t="n">
+        <v>0</v>
+      </c>
       <c r="F90" s="119" t="n"/>
       <c r="G90" s="119" t="n"/>
       <c r="H90" s="119" t="n"/>
@@ -15834,7 +15834,7 @@
       <c r="N90" s="119" t="n"/>
       <c r="O90" s="119" t="n"/>
       <c r="P90" s="119" t="n">
-        <v>4269.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" ht="35.25" customHeight="1" s="134">
@@ -15853,10 +15853,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D91" s="116" t="n">
-        <v>0</v>
-      </c>
-      <c r="E91" s="116" t="n"/>
+      <c r="D91" s="116" t="n"/>
+      <c r="E91" s="116" t="n">
+        <v>48970.67</v>
+      </c>
       <c r="F91" s="116" t="n"/>
       <c r="G91" s="116" t="n"/>
       <c r="H91" s="116" t="n"/>
@@ -15868,7 +15868,7 @@
       <c r="N91" s="116" t="n"/>
       <c r="O91" s="116" t="n"/>
       <c r="P91" s="116" t="n">
-        <v>0</v>
+        <v>48970.67</v>
       </c>
     </row>
     <row r="92" ht="35.25" customHeight="1" s="134">
@@ -15887,10 +15887,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D92" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="E92" s="119" t="n"/>
+      <c r="D92" s="119" t="n"/>
+      <c r="E92" s="119" t="n">
+        <v>48970.67</v>
+      </c>
       <c r="F92" s="119" t="n"/>
       <c r="G92" s="119" t="n"/>
       <c r="H92" s="119" t="n"/>
@@ -15902,7 +15902,7 @@
       <c r="N92" s="119" t="n"/>
       <c r="O92" s="119" t="n"/>
       <c r="P92" s="119" t="n">
-        <v>0</v>
+        <v>48970.67</v>
       </c>
     </row>
     <row r="93" ht="35.25" customHeight="1" s="134">
@@ -15921,10 +15921,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D93" s="119" t="n">
+      <c r="D93" s="119" t="n"/>
+      <c r="E93" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E93" s="119" t="n"/>
       <c r="F93" s="119" t="n"/>
       <c r="G93" s="119" t="n"/>
       <c r="H93" s="119" t="n"/>
@@ -15955,10 +15955,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D94" s="116" t="n">
-        <v>10317.24</v>
-      </c>
-      <c r="E94" s="116" t="n"/>
+      <c r="D94" s="116" t="n"/>
+      <c r="E94" s="116" t="n">
+        <v>0</v>
+      </c>
       <c r="F94" s="116" t="n"/>
       <c r="G94" s="116" t="n"/>
       <c r="H94" s="116" t="n"/>
@@ -15970,7 +15970,7 @@
       <c r="N94" s="116" t="n"/>
       <c r="O94" s="116" t="n"/>
       <c r="P94" s="116" t="n">
-        <v>10317.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" ht="35.25" customHeight="1" s="134">
@@ -15989,10 +15989,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D95" s="119" t="n">
+      <c r="D95" s="119" t="n"/>
+      <c r="E95" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E95" s="119" t="n"/>
       <c r="F95" s="119" t="n"/>
       <c r="G95" s="119" t="n"/>
       <c r="H95" s="119" t="n"/>
@@ -16023,10 +16023,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D96" s="119" t="n">
-        <v>10317.24</v>
-      </c>
-      <c r="E96" s="119" t="n"/>
+      <c r="D96" s="119" t="n"/>
+      <c r="E96" s="119" t="n">
+        <v>0</v>
+      </c>
       <c r="F96" s="119" t="n"/>
       <c r="G96" s="119" t="n"/>
       <c r="H96" s="119" t="n"/>
@@ -16038,7 +16038,7 @@
       <c r="N96" s="119" t="n"/>
       <c r="O96" s="119" t="n"/>
       <c r="P96" s="119" t="n">
-        <v>10317.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" ht="35.25" customHeight="1" s="134">
@@ -16057,10 +16057,10 @@
           <t>Total requalificado (m2)</t>
         </is>
       </c>
-      <c r="D97" s="116" t="n">
+      <c r="D97" s="116" t="n"/>
+      <c r="E97" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="E97" s="116" t="n"/>
       <c r="F97" s="116" t="n"/>
       <c r="G97" s="116" t="n"/>
       <c r="H97" s="116" t="n"/>
@@ -16091,10 +16091,10 @@
           <t>SMSUB/CONVIAS</t>
         </is>
       </c>
-      <c r="D98" s="119" t="n">
+      <c r="D98" s="119" t="n"/>
+      <c r="E98" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E98" s="119" t="n"/>
       <c r="F98" s="119" t="n"/>
       <c r="G98" s="119" t="n"/>
       <c r="H98" s="119" t="n"/>
@@ -16125,10 +16125,10 @@
           <t>SMSUB/CONSEMAVI</t>
         </is>
       </c>
-      <c r="D99" s="119" t="n">
+      <c r="D99" s="119" t="n"/>
+      <c r="E99" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="E99" s="119" t="n"/>
       <c r="F99" s="119" t="n"/>
       <c r="G99" s="119" t="n"/>
       <c r="H99" s="119" t="n"/>
@@ -16152,10 +16152,10 @@
       <c r="B100" s="138" t="n"/>
       <c r="C100" s="136" t="n"/>
       <c r="D100" s="121" t="n">
-        <v>72870.70000000001</v>
+        <v>0</v>
       </c>
       <c r="E100" s="121" t="n">
-        <v>0</v>
+        <v>182420.4</v>
       </c>
       <c r="F100" s="121" t="n">
         <v>0</v>
@@ -16188,7 +16188,7 @@
         <v>0</v>
       </c>
       <c r="P100" s="121" t="n">
-        <v>72870.70000000001</v>
+        <v>182420.4</v>
       </c>
     </row>
     <row r="101" ht="35.25" customHeight="1" s="134">

</xml_diff>